<commit_message>
SISTEMA SEM DESCONTO NA PLANILHA DE EMISSÃO
</commit_message>
<xml_diff>
--- a/envio_rendimentos/arquivos_gerados/EMPRESAS_NOMECURTO_CNPJ.xlsx
+++ b/envio_rendimentos/arquivos_gerados/EMPRESAS_NOMECURTO_CNPJ.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29009"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PGC\envio_rendimentos\arquivos_gerados\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PGC\envio_rendimentos\arquivos_gerados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1585ACD-07A1-4B54-9150-16254FDB8A6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C606725-8F7F-4980-AF85-2C278A3A4E75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{9C6E5FCC-DFCE-4D73-A9A7-EAE5958E03F6}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9C6E5FCC-DFCE-4D73-A9A7-EAE5958E03F6}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="25">
   <si>
     <t>34.028.040/0003-25</t>
   </si>
@@ -93,6 +93,24 @@
   </si>
   <si>
     <t>72 - CANELA EMPREENDIMENTOS IMOBILIARIOS LTDA</t>
+  </si>
+  <si>
+    <t>6 - LGM PARTICIPACOES LTDA | FILIAL BORGES</t>
+  </si>
+  <si>
+    <t>48.896.217/0004-09</t>
+  </si>
+  <si>
+    <t>16 - LSRG RESORT SPE LTDA SCP</t>
+  </si>
+  <si>
+    <t>17 - SCI RESORT SPE LTDA SCP</t>
+  </si>
+  <si>
+    <t>49.850.335/0001-98</t>
+  </si>
+  <si>
+    <t>49.729.088/0001-76</t>
   </si>
 </sst>
 </file>
@@ -473,11 +491,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE962F03-3E72-4606-9A8A-3FFD8B6A38D9}">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="58.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="58.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -505,82 +522,119 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C5" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C6" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C8" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C9" t="s">
-        <v>7</v>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C9">
+    <sortCondition ref="A1:A9"/>
+  </sortState>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>